<commit_message>
🐛 FIX CRÍTICO: Validación y corrección de factorTemperatura + logging detallado
- Detecta si factorTemperatura está en formato porcentual (>1.0) y lo corrige automáticamente dividiendo /100
- Valida rango válido (0.5-1.0) en ambas funciones de cálculo
- Agrega logging detallado para diagnosticar cálculos de generación
- Muestra todos los parámetros del cálculo: consumo, equipos, HSP, factorTemp, energía por panel, número de paneles
- Alerta cuando generación mensual > 10x consumo (posible error)
- Implementado en calcular_cotizacion() y calcular_segunda_opcion()

Este fix resuelve el bug de generación excesiva (133056 kWh para 1000 kWh consumo)
</commit_message>
<xml_diff>
--- a/Modificaciones al cotizador.xlsx
+++ b/Modificaciones al cotizador.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="46">
   <si>
     <t>COTIZADOR FOTOVOLTAICO</t>
   </si>
@@ -53,6 +53,9 @@
     <t>Se resume en dos lineas</t>
   </si>
   <si>
+    <t>APLICADA</t>
+  </si>
+  <si>
     <t>Los servicios puntuales comienzan con palabras  similares</t>
   </si>
   <si>
@@ -62,12 +65,18 @@
     <t>Eliminamos el acopañamiento de Medidor</t>
   </si>
   <si>
+    <t>aplicado</t>
+  </si>
+  <si>
     <t>Se modificó la descripción de los datos suministrados por el cliente.</t>
   </si>
   <si>
     <t>COLORES DEL FORMATO DE COTIZACION PPTX</t>
   </si>
   <si>
+    <t>luisfer</t>
+  </si>
+  <si>
     <t>Cómo utilizar la informción uso de la energía: Diurno/Nocturno</t>
   </si>
   <si>
@@ -77,9 +86,6 @@
     <t>Se elimina el ícono de la solución ppropuesta</t>
   </si>
   <si>
-    <t>APLICADA</t>
-  </si>
-  <si>
     <t>Cuando no hay Baterías en el solución, debe eliminarse esa linea o quitar los paréntesis</t>
   </si>
   <si>
@@ -101,6 +107,9 @@
     <t>CORREGIR LA MINIMA AREA DE ESPACIO PARA INSTALACION DE PANELES</t>
   </si>
   <si>
+    <t>???</t>
+  </si>
+  <si>
     <t>Cuando el nro de pisos supere los 4, permitir e¿que el usuario digite el numero de pisos</t>
   </si>
   <si>
@@ -113,7 +122,49 @@
     <t>Enviar el correo después de verificar en pantalla los siguientes datos: Precio uniotario y total de cada item, valor de IVA, etc tec</t>
   </si>
   <si>
-    <t xml:space="preserve">Verificar ortografía de valores y textos de toda la cotización. </t>
+    <t>Verificar ortografía de los valores de las variables y del texto de la plantilla. bifasico, etc</t>
+  </si>
+  <si>
+    <t>No aplicado</t>
+  </si>
+  <si>
+    <t>El número de la cotización que sea consecutivo. ?????</t>
+  </si>
+  <si>
+    <t>Crear un formato en TABLA_AHORROS para que el signo $ quede siempre alineado a la derecha y no se pegue al valor.</t>
+  </si>
+  <si>
+    <t>En proceso</t>
+  </si>
+  <si>
+    <t>Adicionar el campo factor de temperatura a ciudad</t>
+  </si>
+  <si>
+    <t>Adicionar trers campos a Inversor; Tipo (String/Micro), Número de canales, sobredimensionamiento</t>
+  </si>
+  <si>
+    <t>Formula para el número de inversores MIcro = numero de paneles / numero canales</t>
+  </si>
+  <si>
+    <t>Formula para el número de inversores String = Capacidad instalada / capacidadInversor*sobredimensionamiento</t>
+  </si>
+  <si>
+    <t>Mostrar los PDFs antes de enviar al cliente. El usuario confirma o cancela el envío.</t>
+  </si>
+  <si>
+    <t>Cuando el nro de inversores caculados no es número entero, debe ajustarse de acuerdo al redondeo y si se ajusta al entero hacia abajo, debe redefinirse el numero de páneles y todo lo que afecta este cambio, si es hacia arriba no se ajusta nada porque los inversores soportarían la capacidad instalada.</t>
+  </si>
+  <si>
+    <t>Adicionar al formulario de captura de datos el campo de POrcentaje de ahorro requerido. Este disminuye la capacidad  requerida de consumo para calcular el sistema.</t>
+  </si>
+  <si>
+    <t>Revisar el archivo de estadistica generado en Backend y los valores por default</t>
+  </si>
+  <si>
+    <t>Cuando se selecciona SI en legalización, debe incluirse un texto que comience por "Gestión ante operador de red......." ver excel</t>
+  </si>
+  <si>
+    <t>Revisar la utilización de Bases de datos</t>
   </si>
 </sst>
 </file>
@@ -1027,8 +1078,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A4:D23" totalsRowShown="0">
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A4:D23" etc:filterBottomFollowUsedRange="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A4:D39" totalsRowShown="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A4:D39" etc:filterBottomFollowUsedRange="0"/>
   <tableColumns count="4">
     <tableColumn id="1" name="NRO"/>
     <tableColumn id="2" name="OBSERVACIONES/MODIF"/>
@@ -1297,11 +1348,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="3"/>
   <cols>
-    <col min="1" max="1" width="6.6328125" customWidth="1"/>
-    <col min="2" max="2" width="35.28125" customWidth="1"/>
+    <col min="1" max="1" width="8.5859375" customWidth="1"/>
+    <col min="2" max="2" width="59.3671875" customWidth="1"/>
     <col min="3" max="3" width="41.6640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1329,7 +1380,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" ht="17" spans="1:3">
+    <row r="5" ht="17" spans="1:4">
       <c r="A5" s="1">
         <v>1</v>
       </c>
@@ -1339,131 +1390,234 @@
       <c r="C5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" ht="34" spans="1:3">
+      <c r="D5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" ht="34" spans="1:4">
       <c r="A6">
         <v>2</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" t="s">
         <v>8</v>
       </c>
-      <c r="C6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" ht="17" spans="1:2">
+    </row>
+    <row r="7" ht="17" spans="1:4">
       <c r="A7">
         <v>3</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" ht="34" spans="1:2">
+        <v>11</v>
+      </c>
+      <c r="D7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" ht="34" spans="1:4">
       <c r="A8">
         <v>4</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
+      </c>
+      <c r="D8" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="2:2">
       <c r="B9" s="2"/>
     </row>
-    <row r="10" ht="34" spans="2:2">
+    <row r="10" ht="34" spans="2:4">
       <c r="B10" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" ht="34" spans="2:3">
+        <v>14</v>
+      </c>
+      <c r="D10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" ht="34" spans="2:4">
       <c r="B11" s="2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C11" t="s">
-        <v>14</v>
+        <v>17</v>
+      </c>
+      <c r="D11" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="12" ht="34" spans="2:4">
       <c r="B12" s="2" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D12" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" ht="51" spans="2:4">
       <c r="B13" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D13" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" ht="51" spans="1:4">
       <c r="A14" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B14" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" ht="34" spans="1:4">
+      <c r="A15" s="3"/>
+      <c r="B15" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" ht="34" spans="1:4">
+      <c r="A16" s="3"/>
+      <c r="B16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4">
+      <c r="B17" s="2"/>
+      <c r="D17" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" ht="34" spans="2:4">
+      <c r="B18" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D18" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" ht="51" spans="2:2">
+      <c r="B19" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" ht="68" spans="2:4">
+      <c r="B20" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D20" t="s">
         <v>20</v>
       </c>
-      <c r="D14" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D15" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D16" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="4:4">
-      <c r="D17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="2:2">
-      <c r="B18" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="19" spans="2:2">
-      <c r="B19" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="20" spans="2:2">
-      <c r="B20" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="21" spans="2:2">
-      <c r="B21" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="22" spans="2:2">
-      <c r="B22" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="23" spans="2:2">
-      <c r="B23" t="s">
-        <v>28</v>
+    </row>
+    <row r="21" ht="34" spans="2:4">
+      <c r="B21" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D21" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" ht="68" spans="2:4">
+      <c r="B22" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D22" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" ht="34" spans="2:4">
+      <c r="B23" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D23" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" ht="34" spans="2:4">
+      <c r="B24" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D24" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="25" ht="51" spans="2:4">
+      <c r="B25" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D25" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="26" ht="34" spans="2:4">
+      <c r="B26" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D26" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27" ht="51" spans="2:2">
+      <c r="B27" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="28" ht="51" spans="2:2">
+      <c r="B28" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="29" ht="51" spans="2:2">
+      <c r="B29" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="30" ht="34" spans="2:2">
+      <c r="B30" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="31" ht="84" spans="2:2">
+      <c r="B31" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="32" ht="84" spans="2:2">
+      <c r="B32" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="33" ht="34" spans="2:2">
+      <c r="B33" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="34" ht="34" spans="2:2">
+      <c r="B34" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="35" ht="17" spans="2:2">
+      <c r="B35" s="2" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>